<commit_message>
CPO692/EPO18 직접 값 반영 16:37
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260424.xlsx
+++ b/RNR_수입원가_2026_20260424.xlsx
@@ -3489,24 +3489,20 @@
       <c r="H19" s="7" t="n">
         <v>11000</v>
       </c>
-      <c r="I19" s="119">
-        <f>IFERROR(VLOOKUP(B19,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I19" s="119" t="n">
+        <v>1482.8</v>
       </c>
       <c r="J19" s="9" t="n">
         <v>16310800</v>
       </c>
-      <c r="K19" s="9">
-        <f>IFERROR(ROUND(H19*I19,0),0)</f>
-        <v/>
-      </c>
-      <c r="L19" s="9">
-        <f>IFERROR(VLOOKUP(B19,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M19" s="9">
-        <f>IFERROR(VLOOKUP(B19,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+      <c r="K19" s="9" t="n">
+        <v>16310800</v>
+      </c>
+      <c r="L19" s="9" t="n">
+        <v>462</v>
+      </c>
+      <c r="M19" s="9" t="n">
+        <v>296</v>
       </c>
       <c r="N19" s="3" t="inlineStr">
         <is>
@@ -3560,16 +3556,14 @@
         <f>S19+T19+W19</f>
         <v/>
       </c>
-      <c r="AA19" s="10">
-        <f>K19+L19+M19+IFERROR(VLOOKUP(B19,RemitTable2,9,FALSE()),0)+Y19+Z19</f>
-        <v/>
+      <c r="AA19" s="10" t="n">
+        <v>20915590</v>
       </c>
       <c r="AB19" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="AC19" s="10">
-        <f>ROUND(AA19/AB19,0)</f>
-        <v/>
+      <c r="AC19" s="10" t="n">
+        <v>10457795</v>
       </c>
       <c r="AD19" s="3" t="inlineStr">
         <is>
@@ -3620,24 +3614,20 @@
       <c r="H20" s="7" t="n">
         <v>286580</v>
       </c>
-      <c r="I20" s="119">
-        <f>IFERROR(VLOOKUP(B20,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I20" s="119" t="n">
+        <v>1482.8</v>
       </c>
       <c r="J20" s="9" t="n">
         <v>424990980</v>
       </c>
-      <c r="K20" s="9">
-        <f>IFERROR(ROUND(H20*I20,0),0)</f>
-        <v/>
-      </c>
-      <c r="L20" s="9">
-        <f>IFERROR(VLOOKUP(B20,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M20" s="9">
-        <f>IFERROR(VLOOKUP(B20,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+      <c r="K20" s="9" t="n">
+        <v>424990980</v>
+      </c>
+      <c r="L20" s="9" t="n">
+        <v>12038</v>
+      </c>
+      <c r="M20" s="9" t="n">
+        <v>7704</v>
       </c>
       <c r="N20" s="3" t="inlineStr">
         <is>
@@ -3691,16 +3681,14 @@
         <f>S20+T20+W20</f>
         <v/>
       </c>
-      <c r="AA20" s="10">
-        <f>K20+L20+M20+IFERROR(VLOOKUP(B20,RemitTable2,9,FALSE()),0)+Y20+Z20</f>
-        <v/>
+      <c r="AA20" s="10" t="n">
+        <v>473718807</v>
       </c>
       <c r="AB20" s="11" t="n">
         <v>28</v>
       </c>
-      <c r="AC20" s="10">
-        <f>ROUND(AA20/AB20,0)</f>
-        <v/>
+      <c r="AC20" s="10" t="n">
+        <v>16918529</v>
       </c>
       <c r="AD20" s="3" t="inlineStr">
         <is>
@@ -5031,24 +5019,20 @@
       <c r="H31" s="125" t="n">
         <v>4388.4</v>
       </c>
-      <c r="I31" s="126">
-        <f>IFERROR(VLOOKUP(B31,RemitTable2,7,FALSE()),0)</f>
-        <v/>
+      <c r="I31" s="126" t="n">
+        <v>1741.08</v>
       </c>
       <c r="J31" s="127" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="127">
-        <f>IFERROR(ROUND(H31*I31,0),0)</f>
-        <v/>
-      </c>
-      <c r="L31" s="127">
-        <f>IFERROR(VLOOKUP(B31,RemitTable2,10,FALSE()),0)</f>
-        <v/>
-      </c>
-      <c r="M31" s="127">
-        <f>IFERROR(VLOOKUP(B31,RemitTable2,11,FALSE()),0)</f>
-        <v/>
+        <v>7702082</v>
+      </c>
+      <c r="K31" s="127" t="n">
+        <v>7702082</v>
+      </c>
+      <c r="L31" s="127" t="n">
+        <v>10000</v>
+      </c>
+      <c r="M31" s="127" t="n">
+        <v>8000</v>
       </c>
       <c r="N31" s="123" t="inlineStr">
         <is>
@@ -5100,16 +5084,14 @@
         <f>S31+T31+W31</f>
         <v/>
       </c>
-      <c r="AA31" s="128">
-        <f>K31+L31+M31+IFERROR(VLOOKUP(B31,RemitTable2,9,FALSE()),0)+Y31+Z31</f>
-        <v/>
+      <c r="AA31" s="128" t="n">
+        <v>7763609</v>
       </c>
       <c r="AB31" s="129" t="n">
         <v>60</v>
       </c>
-      <c r="AC31" s="128">
-        <f>ROUND(AA31/AB31,0)</f>
-        <v/>
+      <c r="AC31" s="128" t="n">
+        <v>129393</v>
       </c>
       <c r="AD31" s="123" t="inlineStr">
         <is>
@@ -10535,7 +10517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M79"/>
+  <dimension ref="A1:M76"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="17"/>
   <cols>
     <col width="12.83203125" customWidth="1" style="107" min="1" max="1"/>
@@ -13770,19 +13752,9 @@
         <v>7763609</v>
       </c>
     </row>
-    <row r="69"/>
-    <row r="70"/>
-    <row r="71"/>
-    <row r="72"/>
-    <row r="73"/>
-    <row r="74"/>
-    <row r="75"/>
     <row r="76">
       <c r="M76" s="56" t="n"/>
     </row>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A33:L33"/>

</xml_diff>

<commit_message>
Update RNR_수입원가_2026_20260424.xlsx 2026-04-24 16:50
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260424.xlsx
+++ b/RNR_수입원가_2026_20260424.xlsx
@@ -24,7 +24,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -32,6 +32,7 @@
     <numFmt numFmtId="168" formatCode="0&quot;일&quot;"/>
     <numFmt numFmtId="169" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="170" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="171" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -406,7 +407,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="181">
+  <cellXfs count="192">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -927,6 +928,39 @@
     </xf>
     <xf numFmtId="165" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="17" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="171" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -8435,7 +8469,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15.75" customHeight="1">
+    <row r="3" ht="16" customHeight="1">
       <c r="A3" s="21" t="n">
         <v>1</v>
       </c>
@@ -8462,25 +8496,17 @@
           <t>EW CP2220</t>
         </is>
       </c>
-      <c r="G3" s="21" t="inlineStr">
-        <is>
-          <t>2025-09-25</t>
-        </is>
-      </c>
-      <c r="H3" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="I3" s="21" t="inlineStr">
-        <is>
-          <t>2025-09-13</t>
-        </is>
-      </c>
-      <c r="J3" s="21" t="inlineStr">
-        <is>
-          <t>2026-08-28</t>
-        </is>
+      <c r="G3" s="190" t="n">
+        <v>45925</v>
+      </c>
+      <c r="H3" s="190" t="n">
+        <v>46080</v>
+      </c>
+      <c r="I3" s="190" t="n">
+        <v>45913</v>
+      </c>
+      <c r="J3" s="190" t="n">
+        <v>46262</v>
       </c>
       <c r="K3" s="21" t="inlineStr">
         <is>
@@ -8488,7 +8514,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="15.75" customHeight="1">
+    <row r="4" ht="16" customHeight="1">
       <c r="A4" s="21" t="n">
         <v>2</v>
       </c>
@@ -8515,25 +8541,17 @@
           <t>HFR License</t>
         </is>
       </c>
-      <c r="G4" s="21" t="inlineStr">
-        <is>
-          <t>2025-11-21</t>
-        </is>
-      </c>
-      <c r="H4" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-23</t>
-        </is>
-      </c>
-      <c r="I4" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-01</t>
-        </is>
-      </c>
-      <c r="J4" s="21" t="inlineStr">
-        <is>
-          <t>2026-11-30</t>
-        </is>
+      <c r="G4" s="190" t="n">
+        <v>45982</v>
+      </c>
+      <c r="H4" s="190" t="n">
+        <v>46014</v>
+      </c>
+      <c r="I4" s="190" t="n">
+        <v>45992</v>
+      </c>
+      <c r="J4" s="190" t="n">
+        <v>46356</v>
       </c>
       <c r="K4" s="21" t="inlineStr">
         <is>
@@ -8541,7 +8559,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="15.75" customHeight="1">
+    <row r="5" ht="16" customHeight="1">
       <c r="A5" s="21" t="n">
         <v>3</v>
       </c>
@@ -8568,25 +8586,17 @@
           <t>EW CP2309/2315/2320-RGB</t>
         </is>
       </c>
-      <c r="G5" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-02</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-11</t>
-        </is>
-      </c>
-      <c r="I5" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-22</t>
-        </is>
-      </c>
-      <c r="J5" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-21</t>
-        </is>
+      <c r="G5" s="190" t="n">
+        <v>45993</v>
+      </c>
+      <c r="H5" s="190" t="n">
+        <v>46064</v>
+      </c>
+      <c r="I5" s="190" t="n">
+        <v>46013</v>
+      </c>
+      <c r="J5" s="190" t="n">
+        <v>46377</v>
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
@@ -8594,7 +8604,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="15.75" customHeight="1">
+    <row r="6" ht="16" customHeight="1">
       <c r="A6" s="21" t="n">
         <v>4</v>
       </c>
@@ -8621,25 +8631,17 @@
           <t>TMS-2000 EW</t>
         </is>
       </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="I6" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J6" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G6" s="190" t="n">
+        <v>46007</v>
+      </c>
+      <c r="H6" s="190" t="n">
+        <v>46043</v>
+      </c>
+      <c r="I6" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J6" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
@@ -8647,7 +8649,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="15.75" customHeight="1">
+    <row r="7" ht="16" customHeight="1">
       <c r="A7" s="21" t="n">
         <v>5</v>
       </c>
@@ -8674,25 +8676,17 @@
           <t>TMS-1000 EW</t>
         </is>
       </c>
-      <c r="G7" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-16</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-21</t>
-        </is>
-      </c>
-      <c r="I7" s="21" t="inlineStr">
-        <is>
-          <t>2025-11-01</t>
-        </is>
-      </c>
-      <c r="J7" s="21" t="inlineStr">
-        <is>
-          <t>2026-10-30</t>
-        </is>
+      <c r="G7" s="190" t="n">
+        <v>46007</v>
+      </c>
+      <c r="H7" s="190" t="n">
+        <v>46043</v>
+      </c>
+      <c r="I7" s="190" t="n">
+        <v>45962</v>
+      </c>
+      <c r="J7" s="190" t="n">
+        <v>46325</v>
       </c>
       <c r="K7" s="21" t="inlineStr">
         <is>
@@ -8700,7 +8694,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="15.75" customHeight="1">
+    <row r="8" ht="16" customHeight="1">
       <c r="A8" s="21" t="n">
         <v>6</v>
       </c>
@@ -8727,25 +8721,17 @@
           <t>EW 대량 (CP2208~CP4450)</t>
         </is>
       </c>
-      <c r="G8" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
-      </c>
-      <c r="H8" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="I8" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J8" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G8" s="190" t="n">
+        <v>46010</v>
+      </c>
+      <c r="H8" s="190" t="n">
+        <v>46080</v>
+      </c>
+      <c r="I8" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J8" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K8" s="21" t="inlineStr">
         <is>
@@ -8753,7 +8739,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1">
+    <row r="9" ht="16" customHeight="1">
       <c r="A9" s="21" t="n">
         <v>7</v>
       </c>
@@ -8780,25 +8766,19 @@
           <t>EW 대량 (SR/SX/TMS)</t>
         </is>
       </c>
-      <c r="G9" s="21" t="inlineStr">
-        <is>
-          <t>2025-12-24</t>
-        </is>
+      <c r="G9" s="190" t="n">
+        <v>46015</v>
       </c>
       <c r="H9" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I9" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J9" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="I9" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J9" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K9" s="21" t="inlineStr">
         <is>
@@ -8806,7 +8786,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15.75" customHeight="1">
+    <row r="10" ht="16" customHeight="1">
       <c r="A10" s="21" t="n">
         <v>8</v>
       </c>
@@ -8833,25 +8813,17 @@
           <t>EW CP2315/CP4440-RGB</t>
         </is>
       </c>
-      <c r="G10" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
-      </c>
-      <c r="H10" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="I10" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="J10" s="21" t="inlineStr">
-        <is>
-          <t>2027-01-29</t>
-        </is>
+      <c r="G10" s="190" t="n">
+        <v>46029</v>
+      </c>
+      <c r="H10" s="190" t="n">
+        <v>46072</v>
+      </c>
+      <c r="I10" s="190" t="n">
+        <v>46052</v>
+      </c>
+      <c r="J10" s="190" t="n">
+        <v>46416</v>
       </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
@@ -8859,7 +8831,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15.75" customHeight="1">
+    <row r="11" ht="16" customHeight="1">
       <c r="A11" s="21" t="n">
         <v>9</v>
       </c>
@@ -8886,10 +8858,8 @@
           <t>EW (홀딩)</t>
         </is>
       </c>
-      <c r="G11" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-07</t>
-        </is>
+      <c r="G11" s="190" t="n">
+        <v>46029</v>
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
@@ -8912,7 +8882,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15.75" customHeight="1">
+    <row r="12" ht="16" customHeight="1">
       <c r="A12" s="21" t="n">
         <v>10</v>
       </c>
@@ -8939,25 +8909,17 @@
           <t>TMS-2000 License</t>
         </is>
       </c>
-      <c r="G12" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="H12" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="I12" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J12" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G12" s="190" t="n">
+        <v>46042</v>
+      </c>
+      <c r="H12" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="I12" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J12" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K12" s="21" t="inlineStr">
         <is>
@@ -8965,7 +8927,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15.75" customHeight="1">
+    <row r="13" ht="16" customHeight="1">
       <c r="A13" s="21" t="n">
         <v>11</v>
       </c>
@@ -8992,25 +8954,17 @@
           <t>SX/SR EW (CGV/Lotte)</t>
         </is>
       </c>
-      <c r="G13" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="H13" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="I13" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J13" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G13" s="190" t="n">
+        <v>46042</v>
+      </c>
+      <c r="H13" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="I13" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J13" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K13" s="21" t="inlineStr">
         <is>
@@ -9018,7 +8972,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15.75" customHeight="1">
+    <row r="14" ht="16" customHeight="1">
       <c r="A14" s="21" t="n">
         <v>12</v>
       </c>
@@ -9045,25 +8999,17 @@
           <t>SR-1000/SX-3000 EW</t>
         </is>
       </c>
-      <c r="G14" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-20</t>
-        </is>
-      </c>
-      <c r="H14" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="I14" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J14" s="21" t="inlineStr">
-        <is>
-          <t>2026-12-31</t>
-        </is>
+      <c r="G14" s="190" t="n">
+        <v>46042</v>
+      </c>
+      <c r="H14" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="I14" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J14" s="190" t="n">
+        <v>46387</v>
       </c>
       <c r="K14" s="21" t="inlineStr">
         <is>
@@ -9071,7 +9017,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15.75" customHeight="1">
+    <row r="15" ht="16" customHeight="1">
       <c r="A15" s="21" t="n">
         <v>13</v>
       </c>
@@ -9098,25 +9044,17 @@
           <t>EW (메가박스 외)</t>
         </is>
       </c>
-      <c r="G15" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-04</t>
-        </is>
-      </c>
-      <c r="H15" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I15" s="21" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="J15" s="95" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="G15" s="190" t="n">
+        <v>46057</v>
+      </c>
+      <c r="H15" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I15" s="190" t="n">
+        <v>46082</v>
+      </c>
+      <c r="J15" s="191" t="n">
+        <v>46446</v>
       </c>
       <c r="K15" s="21" t="inlineStr">
         <is>
@@ -9124,7 +9062,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1">
+    <row r="16" ht="16" customHeight="1">
       <c r="A16" s="21" t="n">
         <v>14</v>
       </c>
@@ -9151,25 +9089,17 @@
           <t>SR/SX EW (하남미사 외)</t>
         </is>
       </c>
-      <c r="G16" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-07</t>
-        </is>
-      </c>
-      <c r="H16" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I16" s="21" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
-      </c>
-      <c r="J16" s="95" t="inlineStr">
-        <is>
-          <t>2027-02-22</t>
-        </is>
+      <c r="G16" s="190" t="n">
+        <v>46060</v>
+      </c>
+      <c r="H16" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I16" s="190" t="n">
+        <v>46023</v>
+      </c>
+      <c r="J16" s="191" t="n">
+        <v>46440</v>
       </c>
       <c r="K16" s="21" t="inlineStr">
         <is>
@@ -9177,7 +9107,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1">
+    <row r="17" ht="16" customHeight="1">
       <c r="A17" s="21" t="n">
         <v>15</v>
       </c>
@@ -9204,25 +9134,17 @@
           <t>TMS-1000 License</t>
         </is>
       </c>
-      <c r="G17" s="21" t="inlineStr">
-        <is>
-          <t>2026-02-27</t>
-        </is>
-      </c>
-      <c r="H17" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I17" s="21" t="inlineStr">
-        <is>
-          <t>2026-03-01</t>
-        </is>
-      </c>
-      <c r="J17" s="95" t="inlineStr">
-        <is>
-          <t>2027-02-28</t>
-        </is>
+      <c r="G17" s="190" t="n">
+        <v>46080</v>
+      </c>
+      <c r="H17" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I17" s="190" t="n">
+        <v>46082</v>
+      </c>
+      <c r="J17" s="191" t="n">
+        <v>46446</v>
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
@@ -9230,60 +9152,56 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15.75" customHeight="1">
-      <c r="A18" s="39" t="n">
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="95" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="39" t="inlineStr">
+      <c r="B18" s="95" t="inlineStr">
         <is>
           <t>GPO471</t>
         </is>
       </c>
-      <c r="C18" s="92" t="inlineStr">
+      <c r="C18" s="181" t="inlineStr">
         <is>
           <t>GDC</t>
         </is>
       </c>
-      <c r="D18" s="92" t="inlineStr">
+      <c r="D18" s="181" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
       </c>
-      <c r="E18" s="94" t="n">
+      <c r="E18" s="182" t="n">
         <v>500</v>
       </c>
-      <c r="F18" s="39" t="inlineStr">
+      <c r="F18" s="95" t="inlineStr">
         <is>
           <t>Dolby Atmos License</t>
         </is>
       </c>
-      <c r="G18" s="39" t="inlineStr">
-        <is>
-          <t>2026-03-07</t>
-        </is>
-      </c>
-      <c r="H18" s="39" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="I18" s="39" t="inlineStr">
+      <c r="G18" s="191" t="n">
+        <v>46088</v>
+      </c>
+      <c r="H18" s="191" t="n">
+        <v>46113</v>
+      </c>
+      <c r="I18" s="95" t="inlineStr">
         <is>
           <t>미확인</t>
         </is>
       </c>
-      <c r="J18" s="96" t="inlineStr">
+      <c r="J18" s="95" t="inlineStr">
         <is>
           <t>미확인</t>
         </is>
       </c>
-      <c r="K18" s="21" t="inlineStr">
+      <c r="K18" s="95" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="15.75" customHeight="1">
+    <row r="19" ht="16" customHeight="1">
       <c r="A19" s="21" t="n">
         <v>17</v>
       </c>
@@ -9310,25 +9228,19 @@
           <t>EW (CGV 동백 외 Warranty Extension)</t>
         </is>
       </c>
-      <c r="G19" s="21" t="inlineStr">
-        <is>
-          <t>2026-03-28</t>
-        </is>
+      <c r="G19" s="190" t="n">
+        <v>46109</v>
       </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="I19" s="21" t="inlineStr">
-        <is>
-          <t>2026-04-01</t>
-        </is>
-      </c>
-      <c r="J19" s="95" t="inlineStr">
-        <is>
-          <t>2027-03-31</t>
-        </is>
+      <c r="I19" s="190" t="n">
+        <v>46113</v>
+      </c>
+      <c r="J19" s="191" t="n">
+        <v>46477</v>
       </c>
       <c r="K19" s="21" t="inlineStr">
         <is>
@@ -9336,95 +9248,95 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15.75" customHeight="1">
-      <c r="A20" s="150" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="150" t="inlineStr">
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="183" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" s="183" t="inlineStr">
         <is>
           <t>CPO697</t>
         </is>
       </c>
-      <c r="C20" s="151" t="inlineStr">
+      <c r="C20" s="184" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D20" s="151" t="inlineStr">
+      <c r="D20" s="184" t="inlineStr">
         <is>
           <t>워런티(EW)</t>
         </is>
       </c>
-      <c r="E20" s="152" t="n">
+      <c r="E20" s="185" t="n">
         <v>15289</v>
       </c>
-      <c r="F20" s="150" t="inlineStr">
+      <c r="F20" s="183" t="inlineStr">
         <is>
           <t>EW CP4425/CP2308/CP2315/CP2309/CP2320 13대</t>
         </is>
       </c>
-      <c r="G20" s="153" t="n">
+      <c r="G20" s="186" t="n">
         <v>46136</v>
       </c>
-      <c r="H20" s="150" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I20" s="153" t="n">
+      <c r="H20" s="186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I20" s="186" t="n">
         <v>46168</v>
       </c>
-      <c r="J20" s="153" t="n">
+      <c r="J20" s="186" t="n">
         <v>46532</v>
       </c>
-      <c r="K20" s="150" t="inlineStr">
+      <c r="K20" s="183" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
-      <c r="A21" s="150" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="150" t="inlineStr">
+    <row r="21" ht="16" customHeight="1">
+      <c r="A21" s="183" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="183" t="inlineStr">
         <is>
           <t>CPO693-2</t>
         </is>
       </c>
-      <c r="C21" s="151" t="inlineStr">
+      <c r="C21" s="184" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D21" s="151" t="inlineStr">
+      <c r="D21" s="184" t="inlineStr">
         <is>
           <t>워런티(EW)</t>
         </is>
       </c>
-      <c r="E21" s="152" t="n">
+      <c r="E21" s="185" t="n">
         <v>2550</v>
       </c>
-      <c r="F21" s="150" t="inlineStr">
+      <c r="F21" s="183" t="inlineStr">
         <is>
           <t>CP4420-RGB 2년 워런티 (CGV 구미)</t>
         </is>
       </c>
-      <c r="G21" s="153" t="n">
+      <c r="G21" s="186" t="n">
         <v>46133</v>
       </c>
-      <c r="H21" s="150" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I21" s="153" t="n">
+      <c r="H21" s="186" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I21" s="186" t="n">
         <v>46142</v>
       </c>
-      <c r="J21" s="153" t="n">
+      <c r="J21" s="186" t="n">
         <v>46872</v>
       </c>
-      <c r="K21" s="150" t="inlineStr">
+      <c r="K21" s="183" t="inlineStr">
         <is>
           <t>라이센스</t>
         </is>
@@ -10614,185 +10526,185 @@
       </c>
     </row>
     <row r="3" ht="15.75" customHeight="1">
-      <c r="A3" s="39" t="n">
+      <c r="A3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="39" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>2025.12.01</t>
         </is>
       </c>
-      <c r="C3" s="92" t="inlineStr">
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D3" s="39" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>CPO668-3, CPO673</t>
         </is>
       </c>
-      <c r="E3" s="40" t="n">
+      <c r="E3" s="44" t="n">
         <v>35563</v>
       </c>
-      <c r="F3" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" s="39" t="n">
+      <c r="F3" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H3" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="42">
+      <c r="H3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" s="9">
         <f>ROUND((E3+G3)*F3+H3+I3,0)</f>
         <v/>
       </c>
-      <c r="L3" s="43">
+      <c r="L3" s="46">
         <f>J3-K3</f>
         <v/>
       </c>
     </row>
     <row r="4" ht="15.75" customHeight="1">
-      <c r="A4" s="39" t="n">
+      <c r="A4" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="39" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>2025.12.02</t>
         </is>
       </c>
-      <c r="C4" s="92" t="inlineStr">
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>GDC</t>
         </is>
       </c>
-      <c r="D4" s="39" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>GPO-445, 446-1, 447, 448</t>
         </is>
       </c>
-      <c r="E4" s="40" t="n">
+      <c r="E4" s="44" t="n">
         <v>55830</v>
       </c>
-      <c r="F4" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="39" t="n">
+      <c r="F4" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="42">
+      <c r="H4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="9">
         <f>ROUND((E4+G4)*F4+H4+I4,0)</f>
         <v/>
       </c>
-      <c r="L4" s="43">
+      <c r="L4" s="46">
         <f>J4-K4</f>
         <v/>
       </c>
     </row>
     <row r="5" ht="15.75" customHeight="1">
-      <c r="A5" s="39" t="n">
+      <c r="A5" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="39" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t>2025.12.02</t>
         </is>
       </c>
-      <c r="C5" s="92" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>Thali Consulting</t>
         </is>
       </c>
-      <c r="D5" s="39" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>(PO미기재)</t>
         </is>
       </c>
-      <c r="E5" s="40" t="n">
+      <c r="E5" s="44" t="n">
         <v>9247.690000000001</v>
       </c>
-      <c r="F5" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="39" t="n">
+      <c r="F5" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H5" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" s="42">
+      <c r="H5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="9">
         <f>ROUND((E5+G5)*F5+H5+I5,0)</f>
         <v/>
       </c>
-      <c r="L5" s="43">
+      <c r="L5" s="46">
         <f>J5-K5</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="15.75" customHeight="1">
-      <c r="A6" s="39" t="n">
+      <c r="A6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t>2025.12.02</t>
         </is>
       </c>
-      <c r="C6" s="92" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>Christie</t>
         </is>
       </c>
-      <c r="D6" s="39" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>CPO-669</t>
         </is>
       </c>
-      <c r="E6" s="40" t="n">
+      <c r="E6" s="44" t="n">
         <v>7410</v>
       </c>
-      <c r="F6" s="161" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="39" t="n">
+      <c r="F6" s="162" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="H6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="42">
+      <c r="H6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="9">
         <f>ROUND((E6+G6)*F6+H6+I6,0)</f>
         <v/>
       </c>
-      <c r="L6" s="43">
+      <c r="L6" s="46">
         <f>J6-K6</f>
         <v/>
       </c>
@@ -10982,47 +10894,47 @@
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">
-      <c r="A11" s="13" t="n">
+      <c r="A11" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="13" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t>2025.12.19</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>GDC(라이센스)</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>/ROC/라이센스</t>
         </is>
       </c>
-      <c r="E11" s="47" t="n">
+      <c r="E11" s="44" t="n">
         <v>1200</v>
       </c>
-      <c r="F11" s="163" t="n">
+      <c r="F11" s="162" t="n">
         <v>1464.9</v>
       </c>
-      <c r="G11" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="H11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="19">
+      <c r="G11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="9">
         <f>ROUND((E11+G11)*F11+H11+I11,0)</f>
         <v/>
       </c>
-      <c r="L11" s="49">
+      <c r="L11" s="46">
         <f>J11-K11</f>
         <v/>
       </c>
@@ -11718,277 +11630,277 @@
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1">
-      <c r="A27" s="13" t="n">
+      <c r="A27" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>2026.04.14</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>GDC</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>GPO468-1, 472, 468-2</t>
+        </is>
+      </c>
+      <c r="E27" s="44" t="n">
+        <v>57650</v>
+      </c>
+      <c r="F27" s="162" t="n">
+        <v>1481.9</v>
+      </c>
+      <c r="G27" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="H27" s="9" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I27" s="9" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>85481673</v>
+      </c>
+      <c r="K27" s="9">
+        <f>ROUND((E27+G27)*F27+H27+I27,0)</f>
+        <v/>
+      </c>
+      <c r="L27" s="46">
+        <f>J27-K27</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="171" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="13" t="inlineStr">
-        <is>
-          <t>2026.04.14</t>
-        </is>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
-        <is>
-          <t>GDC</t>
-        </is>
-      </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>GPO468-1, 472, 468-2</t>
-        </is>
-      </c>
-      <c r="E27" s="47" t="n">
-        <v>57650</v>
-      </c>
-      <c r="F27" s="163" t="n">
-        <v>1481.9</v>
-      </c>
-      <c r="G27" s="13" t="n">
+      <c r="B28" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.01</t>
+        </is>
+      </c>
+      <c r="C28" s="172" t="inlineStr">
+        <is>
+          <t>Swank</t>
+        </is>
+      </c>
+      <c r="D28" s="171" t="inlineStr">
+        <is>
+          <t>(영화 라이센스)</t>
+        </is>
+      </c>
+      <c r="E28" s="173" t="n">
+        <v>814</v>
+      </c>
+      <c r="F28" s="187" t="n">
+        <v>1505</v>
+      </c>
+      <c r="G28" s="171" t="n">
         <v>20</v>
       </c>
-      <c r="H27" s="19" t="n">
+      <c r="H28" s="176" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I28" s="176" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J28" s="176" t="n">
+        <v>1268170</v>
+      </c>
+      <c r="K28" s="176">
+        <f>ROUND((E28+G28)*F28+H28+I28,0)</f>
+        <v/>
+      </c>
+      <c r="L28" s="177">
+        <f>J28-K28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="27.75" customHeight="1">
+      <c r="A29" s="171" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.02</t>
+        </is>
+      </c>
+      <c r="C29" s="172" t="inlineStr">
+        <is>
+          <t>Monoplex</t>
+        </is>
+      </c>
+      <c r="D29" s="171" t="inlineStr">
+        <is>
+          <t>(영업)</t>
+        </is>
+      </c>
+      <c r="E29" s="173" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F29" s="187" t="n">
+        <v>1520.1</v>
+      </c>
+      <c r="G29" s="171" t="n">
+        <v>20</v>
+      </c>
+      <c r="H29" s="176" t="n">
+        <v>25000</v>
+      </c>
+      <c r="I29" s="176" t="n">
+        <v>8000</v>
+      </c>
+      <c r="J29" s="176" t="n">
+        <v>45666402</v>
+      </c>
+      <c r="K29" s="176">
+        <f>ROUND((E29+G29)*F29+H29+I29,0)</f>
+        <v/>
+      </c>
+      <c r="L29" s="177">
+        <f>J29-K29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="A30" s="171" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.21</t>
+        </is>
+      </c>
+      <c r="C30" s="172" t="inlineStr">
+        <is>
+          <t>Ferco</t>
+        </is>
+      </c>
+      <c r="D30" s="171" t="inlineStr">
+        <is>
+          <t>MONOPLEX20260126-01</t>
+        </is>
+      </c>
+      <c r="E30" s="173" t="n">
+        <v>25976</v>
+      </c>
+      <c r="F30" s="187" t="n">
+        <v>1473.3</v>
+      </c>
+      <c r="G30" s="171" t="n">
+        <v>20</v>
+      </c>
+      <c r="H30" s="176" t="n">
         <v>12500</v>
       </c>
-      <c r="I27" s="19" t="n">
+      <c r="I30" s="176" t="n">
         <v>8000</v>
       </c>
-      <c r="J27" s="19" t="n">
-        <v>85481673</v>
-      </c>
-      <c r="K27" s="19">
-        <f>ROUND((E27+G27)*F27+H27+I27,0)</f>
-        <v/>
-      </c>
-      <c r="L27" s="49">
-        <f>J27-K27</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="164" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.01</t>
-        </is>
-      </c>
-      <c r="C28" s="165" t="inlineStr">
-        <is>
-          <t>Swank</t>
-        </is>
-      </c>
-      <c r="D28" s="164" t="inlineStr">
-        <is>
-          <t>(영화 라이센스)</t>
-        </is>
-      </c>
-      <c r="E28" s="166" t="n">
-        <v>814</v>
-      </c>
-      <c r="F28" s="167" t="n">
-        <v>1505</v>
-      </c>
-      <c r="G28" s="164" t="n">
+      <c r="J30" s="176" t="n">
+        <v>38320406</v>
+      </c>
+      <c r="K30" s="176">
+        <f>ROUND((E30+G30)*F30+H30+I30,0)</f>
+        <v/>
+      </c>
+      <c r="L30" s="177">
+        <f>J30-K30</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="A31" s="171" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.22</t>
+        </is>
+      </c>
+      <c r="C31" s="172" t="inlineStr">
+        <is>
+          <t>Christie</t>
+        </is>
+      </c>
+      <c r="D31" s="171" t="inlineStr">
+        <is>
+          <t>CPO692(692-1, 692-2)</t>
+        </is>
+      </c>
+      <c r="E31" s="173" t="n">
+        <v>297580</v>
+      </c>
+      <c r="F31" s="187" t="n">
+        <v>1482.8</v>
+      </c>
+      <c r="G31" s="171" t="n">
         <v>20</v>
       </c>
-      <c r="H28" s="168" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I28" s="168" t="n">
+      <c r="H31" s="176" t="n">
+        <v>12500</v>
+      </c>
+      <c r="I31" s="176" t="n">
         <v>8000</v>
       </c>
-      <c r="J28" s="168" t="n">
-        <v>1268170</v>
-      </c>
-      <c r="K28" s="168">
-        <f>ROUND((E28+G28)*F28+H28+I28,0)</f>
-        <v/>
-      </c>
-      <c r="L28" s="169">
-        <f>J28-K28</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="27.75" customHeight="1">
-      <c r="A29" s="164" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.02</t>
-        </is>
-      </c>
-      <c r="C29" s="165" t="inlineStr">
-        <is>
-          <t>Monoplex</t>
-        </is>
-      </c>
-      <c r="D29" s="164" t="inlineStr">
-        <is>
-          <t>(영업)</t>
-        </is>
-      </c>
-      <c r="E29" s="166" t="n">
-        <v>30000</v>
-      </c>
-      <c r="F29" s="167" t="n">
-        <v>1520.1</v>
-      </c>
-      <c r="G29" s="164" t="n">
-        <v>20</v>
-      </c>
-      <c r="H29" s="168" t="n">
-        <v>25000</v>
-      </c>
-      <c r="I29" s="168" t="n">
+      <c r="J31" s="176" t="n">
+        <v>441301780</v>
+      </c>
+      <c r="K31" s="176">
+        <f>ROUND((E31+G31)*F31+H31+I31,0)</f>
+        <v/>
+      </c>
+      <c r="L31" s="177">
+        <f>J31-K31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="A32" s="171" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" s="171" t="inlineStr">
+        <is>
+          <t>2026.04.22</t>
+        </is>
+      </c>
+      <c r="C32" s="172" t="inlineStr">
+        <is>
+          <t>Elicent (EUR)</t>
+        </is>
+      </c>
+      <c r="D32" s="171" t="inlineStr">
+        <is>
+          <t>EPO18</t>
+        </is>
+      </c>
+      <c r="E32" s="173" t="n">
+        <v>4388.4</v>
+      </c>
+      <c r="F32" s="187" t="n">
+        <v>1741.08</v>
+      </c>
+      <c r="G32" s="171" t="n">
+        <v>25</v>
+      </c>
+      <c r="H32" s="176" t="n">
+        <v>10000</v>
+      </c>
+      <c r="I32" s="176" t="n">
         <v>8000</v>
       </c>
-      <c r="J29" s="168" t="n">
-        <v>45666402</v>
-      </c>
-      <c r="K29" s="168">
-        <f>ROUND((E29+G29)*F29+H29+I29,0)</f>
-        <v/>
-      </c>
-      <c r="L29" s="169">
-        <f>J29-K29</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="A30" s="164" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.21</t>
-        </is>
-      </c>
-      <c r="C30" s="165" t="inlineStr">
-        <is>
-          <t>Ferco</t>
-        </is>
-      </c>
-      <c r="D30" s="164" t="inlineStr">
-        <is>
-          <t>MONOPLEX20260126-01</t>
-        </is>
-      </c>
-      <c r="E30" s="166" t="n">
-        <v>25976</v>
-      </c>
-      <c r="F30" s="167" t="n">
-        <v>1473.3</v>
-      </c>
-      <c r="G30" s="164" t="n">
-        <v>20</v>
-      </c>
-      <c r="H30" s="168" t="n">
-        <v>12500</v>
-      </c>
-      <c r="I30" s="168" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J30" s="168" t="n">
-        <v>38320406</v>
-      </c>
-      <c r="K30" s="168">
-        <f>ROUND((E30+G30)*F30+H30+I30,0)</f>
-        <v/>
-      </c>
-      <c r="L30" s="169">
-        <f>J30-K30</f>
-        <v/>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="A31" s="164" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.22</t>
-        </is>
-      </c>
-      <c r="C31" s="165" t="inlineStr">
-        <is>
-          <t>Christie</t>
-        </is>
-      </c>
-      <c r="D31" s="164" t="inlineStr">
-        <is>
-          <t>CPO692(692-1, 692-2)</t>
-        </is>
-      </c>
-      <c r="E31" s="166" t="n">
-        <v>297580</v>
-      </c>
-      <c r="F31" s="167" t="n">
-        <v>1482.8</v>
-      </c>
-      <c r="G31" s="164" t="n">
-        <v>20</v>
-      </c>
-      <c r="H31" s="168" t="n">
-        <v>12500</v>
-      </c>
-      <c r="I31" s="168" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J31" s="168" t="n">
-        <v>441301780</v>
-      </c>
-      <c r="K31" s="168">
-        <f>ROUND((E31+G31)*F31+H31+I31,0)</f>
-        <v/>
-      </c>
-      <c r="L31" s="169">
-        <f>J31-K31</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="A32" s="164" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="164" t="inlineStr">
-        <is>
-          <t>2026.04.22</t>
-        </is>
-      </c>
-      <c r="C32" s="165" t="inlineStr">
-        <is>
-          <t>Elicent (EUR)</t>
-        </is>
-      </c>
-      <c r="D32" s="164" t="inlineStr">
-        <is>
-          <t>EPO18</t>
-        </is>
-      </c>
-      <c r="E32" s="166" t="n">
-        <v>4388.4</v>
-      </c>
-      <c r="F32" s="167" t="n">
-        <v>1741.08</v>
-      </c>
-      <c r="G32" s="164" t="n">
-        <v>25</v>
-      </c>
-      <c r="H32" s="168" t="n">
-        <v>10000</v>
-      </c>
-      <c r="I32" s="168" t="n">
-        <v>8000</v>
-      </c>
-      <c r="J32" s="168" t="n">
+      <c r="J32" s="176" t="n">
         <v>7702082</v>
       </c>
-      <c r="K32" s="168">
+      <c r="K32" s="176">
         <f>ROUND((E32+G32)*F32+H32+I32,0)</f>
         <v/>
       </c>
-      <c r="L32" s="169">
+      <c r="L32" s="177">
         <f>J32-K32</f>
         <v/>
       </c>
@@ -12095,31 +12007,32 @@
       <c r="E35" s="44" t="n">
         <v>143557</v>
       </c>
-      <c r="F35" s="170">
-        <f>D30/E30</f>
-        <v/>
-      </c>
-      <c r="G35" s="119" t="n">
-        <v>1479.7</v>
+      <c r="F35" s="188">
+        <f>D35/E35</f>
+        <v/>
+      </c>
+      <c r="G35" s="44">
+        <f>F10</f>
+        <v/>
       </c>
       <c r="H35" s="9">
-        <f>ROUND(D30*G30,0)</f>
+        <f>ROUND(D35*G35,0)</f>
         <v/>
       </c>
       <c r="I35" s="9">
-        <f>ROUND(20*G30*F30,0)</f>
+        <f>ROUND(G10*F35*G35,0)</f>
         <v/>
       </c>
       <c r="J35" s="9">
-        <f>ROUND(H10*F30,0)</f>
+        <f>ROUND(H10*F35,0)</f>
         <v/>
       </c>
       <c r="K35" s="9">
-        <f>ROUND(I10*F30,0)</f>
+        <f>ROUND(I10*F35,0)</f>
         <v/>
       </c>
       <c r="L35" s="46">
-        <f>H30+I30+J30+K30</f>
+        <f>H35+I35+J35+K35</f>
         <v/>
       </c>
     </row>
@@ -12145,31 +12058,32 @@
       <c r="E36" s="44" t="n">
         <v>143557</v>
       </c>
-      <c r="F36" s="170">
-        <f>D31/E31</f>
-        <v/>
-      </c>
-      <c r="G36" s="119" t="n">
-        <v>1479.7</v>
+      <c r="F36" s="188">
+        <f>D36/E36</f>
+        <v/>
+      </c>
+      <c r="G36" s="44">
+        <f>F10</f>
+        <v/>
       </c>
       <c r="H36" s="9">
-        <f>ROUND(D31*G31,0)</f>
+        <f>ROUND(D36*G36,0)</f>
         <v/>
       </c>
       <c r="I36" s="9">
-        <f>ROUND(20*G31*F31,0)</f>
+        <f>ROUND(G10*F36*G36,0)</f>
         <v/>
       </c>
       <c r="J36" s="9">
-        <f>ROUND(H10*F31,0)</f>
+        <f>ROUND(H10*F36,0)</f>
         <v/>
       </c>
       <c r="K36" s="9">
-        <f>ROUND(I10*F31,0)</f>
+        <f>ROUND(I10*F36,0)</f>
         <v/>
       </c>
       <c r="L36" s="46">
-        <f>H31+I31+J31+K31</f>
+        <f>H36+I36+J36+K36</f>
         <v/>
       </c>
     </row>
@@ -12195,31 +12109,32 @@
       <c r="E37" s="44" t="n">
         <v>15040</v>
       </c>
-      <c r="F37" s="170">
-        <f>D32/E32</f>
-        <v/>
-      </c>
-      <c r="G37" s="119" t="n">
-        <v>1480</v>
+      <c r="F37" s="188">
+        <f>D37/E37</f>
+        <v/>
+      </c>
+      <c r="G37" s="44">
+        <f>F9</f>
+        <v/>
       </c>
       <c r="H37" s="9">
-        <f>ROUND(D32*G32,0)</f>
+        <f>ROUND(D37*G37,0)</f>
         <v/>
       </c>
       <c r="I37" s="9">
-        <f>ROUND(20*G32*F32,0)</f>
+        <f>ROUND(G9*F37*G37,0)</f>
         <v/>
       </c>
       <c r="J37" s="9">
-        <f>ROUND(H9*F32,0)</f>
+        <f>ROUND(H9*F37,0)</f>
         <v/>
       </c>
       <c r="K37" s="9">
-        <f>ROUND(I9*F32,0)</f>
+        <f>ROUND(I9*F37,0)</f>
         <v/>
       </c>
       <c r="L37" s="46">
-        <f>H32+I32+J32+K32</f>
+        <f>H37+I37+J37+K37</f>
         <v/>
       </c>
     </row>
@@ -12245,31 +12160,32 @@
       <c r="E38" s="44" t="n">
         <v>13860</v>
       </c>
-      <c r="F38" s="170">
-        <f>D33/E33</f>
-        <v/>
-      </c>
-      <c r="G38" s="119" t="n">
-        <v>1439.1</v>
+      <c r="F38" s="188">
+        <f>D38/E38</f>
+        <v/>
+      </c>
+      <c r="G38" s="44">
+        <f>F12</f>
+        <v/>
       </c>
       <c r="H38" s="9">
-        <f>ROUND(D33*G33,0)</f>
+        <f>ROUND(D38*G38,0)</f>
         <v/>
       </c>
       <c r="I38" s="9">
-        <f>ROUND(20*G33*F33,0)</f>
+        <f>ROUND(G12*F38*G38,0)</f>
         <v/>
       </c>
       <c r="J38" s="9">
-        <f>ROUND(H12*F33,0)</f>
+        <f>ROUND(H12*F38,0)</f>
         <v/>
       </c>
       <c r="K38" s="9">
-        <f>ROUND(I12*F33,0)</f>
+        <f>ROUND(I12*F38,0)</f>
         <v/>
       </c>
       <c r="L38" s="46">
-        <f>H33+I33+J33+K33</f>
+        <f>H38+I38+J38+K38</f>
         <v/>
       </c>
     </row>
@@ -12295,31 +12211,32 @@
       <c r="E39" s="44" t="n">
         <v>13860</v>
       </c>
-      <c r="F39" s="170">
-        <f>D34/E34</f>
-        <v/>
-      </c>
-      <c r="G39" s="119" t="n">
-        <v>1439.1</v>
+      <c r="F39" s="188">
+        <f>D39/E39</f>
+        <v/>
+      </c>
+      <c r="G39" s="44">
+        <f>F12</f>
+        <v/>
       </c>
       <c r="H39" s="9">
-        <f>ROUND(D34*G34,0)</f>
+        <f>ROUND(D39*G39,0)</f>
         <v/>
       </c>
       <c r="I39" s="9">
-        <f>ROUND(20*G34*F34,0)</f>
+        <f>ROUND(G12*F39*G39,0)</f>
         <v/>
       </c>
       <c r="J39" s="9">
-        <f>ROUND(H12*F34,0)</f>
+        <f>ROUND(H12*F39,0)</f>
         <v/>
       </c>
       <c r="K39" s="9">
-        <f>ROUND(I12*F34,0)</f>
+        <f>ROUND(I12*F39,0)</f>
         <v/>
       </c>
       <c r="L39" s="46">
-        <f>H34+I34+J34+K34</f>
+        <f>H39+I39+J39+K39</f>
         <v/>
       </c>
     </row>
@@ -12345,31 +12262,32 @@
       <c r="E40" s="44" t="n">
         <v>252</v>
       </c>
-      <c r="F40" s="170">
-        <f>D35/E35</f>
-        <v/>
-      </c>
-      <c r="G40" s="119" t="n">
-        <v>1479</v>
+      <c r="F40" s="188">
+        <f>D40/E40</f>
+        <v/>
+      </c>
+      <c r="G40" s="44">
+        <f>F14</f>
+        <v/>
       </c>
       <c r="H40" s="9">
-        <f>ROUND(D35*G35,0)</f>
+        <f>ROUND(D40*G40,0)</f>
         <v/>
       </c>
       <c r="I40" s="9">
-        <f>ROUND(20*G35*F35,0)</f>
+        <f>ROUND(G14*F40*G40,0)</f>
         <v/>
       </c>
       <c r="J40" s="9">
-        <f>ROUND(H14*F35,0)</f>
+        <f>ROUND(H14*F40,0)</f>
         <v/>
       </c>
       <c r="K40" s="9">
-        <f>ROUND(I14*F35,0)</f>
+        <f>ROUND(I14*F40,0)</f>
         <v/>
       </c>
       <c r="L40" s="46">
-        <f>H35+I35+J35+K35</f>
+        <f>H40+I40+J40+K40</f>
         <v/>
       </c>
     </row>
@@ -12395,31 +12313,32 @@
       <c r="E41" s="44" t="n">
         <v>3700</v>
       </c>
-      <c r="F41" s="170">
-        <f>D36/E36</f>
-        <v/>
-      </c>
-      <c r="G41" s="119" t="n">
-        <v>1475.7</v>
+      <c r="F41" s="188">
+        <f>D41/E41</f>
+        <v/>
+      </c>
+      <c r="G41" s="44">
+        <f>F15</f>
+        <v/>
       </c>
       <c r="H41" s="9">
-        <f>ROUND(D36*G36,0)</f>
+        <f>ROUND(D41*G41,0)</f>
         <v/>
       </c>
       <c r="I41" s="9">
-        <f>ROUND(20*G36*F36,0)</f>
+        <f>ROUND(G15*F41*G41,0)</f>
         <v/>
       </c>
       <c r="J41" s="9">
-        <f>ROUND(H15*F36,0)</f>
+        <f>ROUND(H15*F41,0)</f>
         <v/>
       </c>
       <c r="K41" s="9">
-        <f>ROUND(I15*F36,0)</f>
+        <f>ROUND(I15*F41,0)</f>
         <v/>
       </c>
       <c r="L41" s="46">
-        <f>H36+I36+J36+K36</f>
+        <f>H41+I41+J41+K41</f>
         <v/>
       </c>
     </row>
@@ -12445,31 +12364,32 @@
       <c r="E42" s="44" t="n">
         <v>3700</v>
       </c>
-      <c r="F42" s="170">
-        <f>D37/E37</f>
-        <v/>
-      </c>
-      <c r="G42" s="119" t="n">
-        <v>1475.7</v>
+      <c r="F42" s="188">
+        <f>D42/E42</f>
+        <v/>
+      </c>
+      <c r="G42" s="44">
+        <f>F15</f>
+        <v/>
       </c>
       <c r="H42" s="9">
-        <f>ROUND(D37*G37,0)</f>
+        <f>ROUND(D42*G42,0)</f>
         <v/>
       </c>
       <c r="I42" s="9">
-        <f>ROUND(20*G37*F37,0)</f>
+        <f>ROUND(G15*F42*G42,0)</f>
         <v/>
       </c>
       <c r="J42" s="9">
-        <f>ROUND(H15*F37,0)</f>
+        <f>ROUND(H15*F42,0)</f>
         <v/>
       </c>
       <c r="K42" s="9">
-        <f>ROUND(I15*F37,0)</f>
+        <f>ROUND(I15*F42,0)</f>
         <v/>
       </c>
       <c r="L42" s="46">
-        <f>H37+I37+J37+K37</f>
+        <f>H42+I42+J42+K42</f>
         <v/>
       </c>
     </row>
@@ -12495,31 +12415,32 @@
       <c r="E43" s="44" t="n">
         <v>3700</v>
       </c>
-      <c r="F43" s="170">
-        <f>D38/E38</f>
-        <v/>
-      </c>
-      <c r="G43" s="119" t="n">
-        <v>1475.7</v>
+      <c r="F43" s="188">
+        <f>D43/E43</f>
+        <v/>
+      </c>
+      <c r="G43" s="44">
+        <f>F15</f>
+        <v/>
       </c>
       <c r="H43" s="9">
-        <f>ROUND(D38*G38,0)</f>
+        <f>ROUND(D43*G43,0)</f>
         <v/>
       </c>
       <c r="I43" s="9">
-        <f>ROUND(20*G38*F38,0)</f>
+        <f>ROUND(G15*F43*G43,0)</f>
         <v/>
       </c>
       <c r="J43" s="9">
-        <f>ROUND(H15*F38,0)</f>
+        <f>ROUND(H15*F43,0)</f>
         <v/>
       </c>
       <c r="K43" s="9">
-        <f>ROUND(I15*F38,0)</f>
+        <f>ROUND(I15*F43,0)</f>
         <v/>
       </c>
       <c r="L43" s="46">
-        <f>H38+I38+J38+K38</f>
+        <f>H43+I43+J43+K43</f>
         <v/>
       </c>
     </row>
@@ -12545,31 +12466,32 @@
       <c r="E44" s="44" t="n">
         <v>9626.35</v>
       </c>
-      <c r="F44" s="170">
-        <f>D39/E39</f>
-        <v/>
-      </c>
-      <c r="G44" s="119" t="n">
-        <v>1476</v>
+      <c r="F44" s="188">
+        <f>D44/E44</f>
+        <v/>
+      </c>
+      <c r="G44" s="44">
+        <f>F16</f>
+        <v/>
       </c>
       <c r="H44" s="9">
-        <f>ROUND(D39*G39,0)</f>
+        <f>ROUND(D44*G44,0)</f>
         <v/>
       </c>
       <c r="I44" s="9">
-        <f>ROUND(20*G39*F39,0)</f>
+        <f>ROUND(G16*F44*G44,0)</f>
         <v/>
       </c>
       <c r="J44" s="9">
-        <f>ROUND(H16*F39,0)</f>
+        <f>ROUND(H16*F44,0)</f>
         <v/>
       </c>
       <c r="K44" s="9">
-        <f>ROUND(I16*F39,0)</f>
+        <f>ROUND(I16*F44,0)</f>
         <v/>
       </c>
       <c r="L44" s="46">
-        <f>H39+I39+J39+K39</f>
+        <f>H44+I44+J44+K44</f>
         <v/>
       </c>
     </row>
@@ -12595,31 +12517,32 @@
       <c r="E45" s="44" t="n">
         <v>5056.8</v>
       </c>
-      <c r="F45" s="170">
-        <f>D40/E40</f>
-        <v/>
-      </c>
-      <c r="G45" s="119" t="n">
-        <v>1445.5</v>
+      <c r="F45" s="188">
+        <f>D45/E45</f>
+        <v/>
+      </c>
+      <c r="G45" s="44">
+        <f>F17</f>
+        <v/>
       </c>
       <c r="H45" s="9">
-        <f>ROUND(D40*G40,0)</f>
+        <f>ROUND(D45*G45,0)</f>
         <v/>
       </c>
       <c r="I45" s="9">
-        <f>ROUND(20*G40*F40,0)</f>
+        <f>ROUND(G17*F45*G45,0)</f>
         <v/>
       </c>
       <c r="J45" s="9">
-        <f>ROUND(H17*F40,0)</f>
+        <f>ROUND(H17*F45,0)</f>
         <v/>
       </c>
       <c r="K45" s="9">
-        <f>ROUND(I17*F40,0)</f>
+        <f>ROUND(I17*F45,0)</f>
         <v/>
       </c>
       <c r="L45" s="46">
-        <f>H40+I40+J40+K40</f>
+        <f>H45+I45+J45+K45</f>
         <v/>
       </c>
     </row>
@@ -12645,31 +12568,32 @@
       <c r="E46" s="44" t="n">
         <v>24794</v>
       </c>
-      <c r="F46" s="170">
-        <f>D41/E41</f>
-        <v/>
-      </c>
-      <c r="G46" s="119" t="n">
-        <v>1454.7</v>
+      <c r="F46" s="188">
+        <f>D46/E46</f>
+        <v/>
+      </c>
+      <c r="G46" s="44">
+        <f>F19</f>
+        <v/>
       </c>
       <c r="H46" s="9">
-        <f>ROUND(D41*G41,0)</f>
+        <f>ROUND(D46*G46,0)</f>
         <v/>
       </c>
       <c r="I46" s="9">
-        <f>ROUND(20*G41*F41,0)</f>
+        <f>ROUND(G19*F46*G46,0)</f>
         <v/>
       </c>
       <c r="J46" s="9">
-        <f>ROUND(H19*F41,0)</f>
+        <f>ROUND(H19*F46,0)</f>
         <v/>
       </c>
       <c r="K46" s="9">
-        <f>ROUND(I19*F41,0)</f>
+        <f>ROUND(I19*F46,0)</f>
         <v/>
       </c>
       <c r="L46" s="46">
-        <f>H41+I41+J41+K41</f>
+        <f>H46+I46+J46+K46</f>
         <v/>
       </c>
     </row>
@@ -12695,31 +12619,32 @@
       <c r="E47" s="44" t="n">
         <v>24794</v>
       </c>
-      <c r="F47" s="170">
-        <f>D42/E42</f>
-        <v/>
-      </c>
-      <c r="G47" s="119" t="n">
-        <v>1454.7</v>
+      <c r="F47" s="188">
+        <f>D47/E47</f>
+        <v/>
+      </c>
+      <c r="G47" s="44">
+        <f>F19</f>
+        <v/>
       </c>
       <c r="H47" s="9">
-        <f>ROUND(D42*G42,0)</f>
+        <f>ROUND(D47*G47,0)</f>
         <v/>
       </c>
       <c r="I47" s="9">
-        <f>ROUND(20*G42*F42,0)</f>
+        <f>ROUND(G19*F47*G47,0)</f>
         <v/>
       </c>
       <c r="J47" s="9">
-        <f>ROUND(H19*F42,0)</f>
+        <f>ROUND(H19*F47,0)</f>
         <v/>
       </c>
       <c r="K47" s="9">
-        <f>ROUND(I19*F42,0)</f>
+        <f>ROUND(I19*F47,0)</f>
         <v/>
       </c>
       <c r="L47" s="46">
-        <f>H42+I42+J42+K42</f>
+        <f>H47+I47+J47+K47</f>
         <v/>
       </c>
     </row>
@@ -12745,31 +12670,32 @@
       <c r="E48" s="44" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F48" s="170">
-        <f>D43/E43</f>
-        <v/>
-      </c>
-      <c r="G48" s="119" t="n">
-        <v>1453.6</v>
+      <c r="F48" s="188">
+        <f>D48/E48</f>
+        <v/>
+      </c>
+      <c r="G48" s="44">
+        <f>F20</f>
+        <v/>
       </c>
       <c r="H48" s="9">
-        <f>ROUND(D43*G43,0)</f>
+        <f>ROUND(D48*G48,0)</f>
         <v/>
       </c>
       <c r="I48" s="9">
-        <f>ROUND(20*G43*F43,0)</f>
+        <f>ROUND(G20*F48*G48,0)</f>
         <v/>
       </c>
       <c r="J48" s="9">
-        <f>ROUND(H20*F43,0)</f>
+        <f>ROUND(H20*F48,0)</f>
         <v/>
       </c>
       <c r="K48" s="9">
-        <f>ROUND(I20*F43,0)</f>
+        <f>ROUND(I20*F48,0)</f>
         <v/>
       </c>
       <c r="L48" s="46">
-        <f>H43+I43+J43+K43</f>
+        <f>H48+I48+J48+K48</f>
         <v/>
       </c>
     </row>
@@ -12795,31 +12721,32 @@
       <c r="E49" s="44" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F49" s="170">
-        <f>D44/E44</f>
-        <v/>
-      </c>
-      <c r="G49" s="119" t="n">
-        <v>1453.6</v>
+      <c r="F49" s="188">
+        <f>D49/E49</f>
+        <v/>
+      </c>
+      <c r="G49" s="44">
+        <f>F20</f>
+        <v/>
       </c>
       <c r="H49" s="9">
-        <f>ROUND(D44*G44,0)</f>
+        <f>ROUND(D49*G49,0)</f>
         <v/>
       </c>
       <c r="I49" s="9">
-        <f>ROUND(20*G44*F44,0)</f>
+        <f>ROUND(G20*F49*G49,0)</f>
         <v/>
       </c>
       <c r="J49" s="9">
-        <f>ROUND(H20*F44,0)</f>
+        <f>ROUND(H20*F49,0)</f>
         <v/>
       </c>
       <c r="K49" s="9">
-        <f>ROUND(I20*F44,0)</f>
+        <f>ROUND(I20*F49,0)</f>
         <v/>
       </c>
       <c r="L49" s="46">
-        <f>H44+I44+J44+K44</f>
+        <f>H49+I49+J49+K49</f>
         <v/>
       </c>
     </row>
@@ -12845,31 +12772,32 @@
       <c r="E50" s="44" t="n">
         <v>11599.57</v>
       </c>
-      <c r="F50" s="170">
-        <f>D45/E45</f>
-        <v/>
-      </c>
-      <c r="G50" s="119" t="n">
-        <v>1453.6</v>
+      <c r="F50" s="188">
+        <f>D50/E50</f>
+        <v/>
+      </c>
+      <c r="G50" s="44">
+        <f>F20</f>
+        <v/>
       </c>
       <c r="H50" s="9">
-        <f>ROUND(D45*G45,0)</f>
+        <f>ROUND(D50*G50,0)</f>
         <v/>
       </c>
       <c r="I50" s="9">
-        <f>ROUND(20*G45*F45,0)</f>
+        <f>ROUND(G20*F50*G50,0)</f>
         <v/>
       </c>
       <c r="J50" s="9">
-        <f>ROUND(H20*F45,0)</f>
+        <f>ROUND(H20*F50,0)</f>
         <v/>
       </c>
       <c r="K50" s="9">
-        <f>ROUND(I20*F45,0)</f>
+        <f>ROUND(I20*F50,0)</f>
         <v/>
       </c>
       <c r="L50" s="46">
-        <f>H45+I45+J45+K45</f>
+        <f>H50+I50+J50+K50</f>
         <v/>
       </c>
     </row>
@@ -12895,31 +12823,32 @@
       <c r="E51" s="44" t="n">
         <v>26358</v>
       </c>
-      <c r="F51" s="170">
-        <f>D46/E46</f>
-        <v/>
-      </c>
-      <c r="G51" s="119" t="n">
-        <v>1460.7</v>
+      <c r="F51" s="188">
+        <f>D51/E51</f>
+        <v/>
+      </c>
+      <c r="G51" s="44">
+        <f>F21</f>
+        <v/>
       </c>
       <c r="H51" s="9">
-        <f>ROUND(D46*G46,0)</f>
+        <f>ROUND(D51*G51,0)</f>
         <v/>
       </c>
       <c r="I51" s="9">
-        <f>ROUND(20*G46*F46,0)</f>
+        <f>ROUND(G21*F51*G51,0)</f>
         <v/>
       </c>
       <c r="J51" s="9">
-        <f>ROUND(H21*F46,0)</f>
+        <f>ROUND(H21*F51,0)</f>
         <v/>
       </c>
       <c r="K51" s="9">
-        <f>ROUND(I21*F46,0)</f>
+        <f>ROUND(I21*F51,0)</f>
         <v/>
       </c>
       <c r="L51" s="46">
-        <f>H46+I46+J46+K46</f>
+        <f>H51+I51+J51+K51</f>
         <v/>
       </c>
     </row>
@@ -12945,31 +12874,32 @@
       <c r="E52" s="44" t="n">
         <v>17538</v>
       </c>
-      <c r="F52" s="170">
-        <f>D47/E47</f>
-        <v/>
-      </c>
-      <c r="G52" s="119" t="n">
-        <v>1451.7</v>
+      <c r="F52" s="188">
+        <f>D52/E52</f>
+        <v/>
+      </c>
+      <c r="G52" s="44">
+        <f>F22</f>
+        <v/>
       </c>
       <c r="H52" s="9">
-        <f>ROUND(D47*G47,0)</f>
+        <f>ROUND(D52*G52,0)</f>
         <v/>
       </c>
       <c r="I52" s="9">
-        <f>ROUND(20*G47*F47,0)</f>
+        <f>ROUND(G22*F52*G52,0)</f>
         <v/>
       </c>
       <c r="J52" s="9">
-        <f>ROUND(H22*F47,0)</f>
+        <f>ROUND(H22*F52,0)</f>
         <v/>
       </c>
       <c r="K52" s="9">
-        <f>ROUND(I22*F47,0)</f>
+        <f>ROUND(I22*F52,0)</f>
         <v/>
       </c>
       <c r="L52" s="46">
-        <f>H47+I47+J47+K47</f>
+        <f>H52+I52+J52+K52</f>
         <v/>
       </c>
     </row>
@@ -12995,30 +12925,34 @@
       <c r="E53" s="44" t="n">
         <v>17538</v>
       </c>
-      <c r="F53" s="170">
-        <f>D48/E48</f>
-        <v/>
-      </c>
-      <c r="G53" s="119" t="n">
-        <v>1451.7</v>
+      <c r="F53" s="188">
+        <f>D53/E53</f>
+        <v/>
+      </c>
+      <c r="G53" s="44">
+        <f>F22</f>
+        <v/>
       </c>
       <c r="H53" s="9">
-        <f>ROUND(D48*G48,0)</f>
+        <f>ROUND(D53*G53,0)</f>
         <v/>
       </c>
       <c r="I53" s="9">
-        <f>ROUND(20*G48*F48,0)</f>
+        <f>ROUND(G22*F53*G53,0)</f>
         <v/>
       </c>
       <c r="J53" s="9">
-        <f>ROUND(H22*F48,0)</f>
+        <f>ROUND(H22*F53,0)</f>
         <v/>
       </c>
       <c r="K53" s="9">
-        <f>ROUND(I22*F48,0)</f>
-        <v/>
-      </c>
-      <c r="L53" s="46" t="n"/>
+        <f>ROUND(I22*F53,0)</f>
+        <v/>
+      </c>
+      <c r="L53" s="46">
+        <f>H53+I53+J53+K53</f>
+        <v/>
+      </c>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
@@ -13042,31 +12976,32 @@
       <c r="E54" s="44" t="n">
         <v>142189</v>
       </c>
-      <c r="F54" s="170">
-        <f>D49/E49</f>
-        <v/>
-      </c>
-      <c r="G54" s="119" t="n">
-        <v>1441.6</v>
+      <c r="F54" s="188">
+        <f>D54/E54</f>
+        <v/>
+      </c>
+      <c r="G54" s="44">
+        <f>F23</f>
+        <v/>
       </c>
       <c r="H54" s="9">
-        <f>ROUND(D49*G49,0)</f>
+        <f>ROUND(D54*G54,0)</f>
         <v/>
       </c>
       <c r="I54" s="9">
-        <f>ROUND(20*G49*F49,0)</f>
+        <f>ROUND(G23*F54*G54,0)</f>
         <v/>
       </c>
       <c r="J54" s="9">
-        <f>ROUND(H23*F49,0)</f>
+        <f>ROUND(H23*F54,0)</f>
         <v/>
       </c>
       <c r="K54" s="9">
-        <f>ROUND(I23*F49,0)</f>
+        <f>ROUND(I23*F54,0)</f>
         <v/>
       </c>
       <c r="L54" s="46">
-        <f>H49+I49+J49+K49</f>
+        <f>H54+I54+J54+K54</f>
         <v/>
       </c>
     </row>
@@ -13092,31 +13027,32 @@
       <c r="E55" s="44" t="n">
         <v>142189</v>
       </c>
-      <c r="F55" s="170">
-        <f>D50/E50</f>
-        <v/>
-      </c>
-      <c r="G55" s="119" t="n">
-        <v>1441.6</v>
+      <c r="F55" s="188">
+        <f>D55/E55</f>
+        <v/>
+      </c>
+      <c r="G55" s="44">
+        <f>F23</f>
+        <v/>
       </c>
       <c r="H55" s="9">
-        <f>ROUND(D50*G50,0)</f>
+        <f>ROUND(D55*G55,0)</f>
         <v/>
       </c>
       <c r="I55" s="9">
-        <f>ROUND(20*G50*F50,0)</f>
+        <f>ROUND(G23*F55*G55,0)</f>
         <v/>
       </c>
       <c r="J55" s="9">
-        <f>ROUND(H23*F50,0)</f>
+        <f>ROUND(H23*F55,0)</f>
         <v/>
       </c>
       <c r="K55" s="9">
-        <f>ROUND(I23*F50,0)</f>
+        <f>ROUND(I23*F55,0)</f>
         <v/>
       </c>
       <c r="L55" s="46">
-        <f>H50+I50+J50+K50</f>
+        <f>H55+I55+J55+K55</f>
         <v/>
       </c>
     </row>
@@ -13142,31 +13078,32 @@
       <c r="E56" s="44" t="n">
         <v>137850</v>
       </c>
-      <c r="F56" s="170">
-        <f>D51/E51</f>
-        <v/>
-      </c>
-      <c r="G56" s="119" t="n">
-        <v>1477.6</v>
+      <c r="F56" s="188">
+        <f>D56/E56</f>
+        <v/>
+      </c>
+      <c r="G56" s="44">
+        <f>F24</f>
+        <v/>
       </c>
       <c r="H56" s="9">
-        <f>ROUND(D51*G51,0)</f>
+        <f>ROUND(D56*G56,0)</f>
         <v/>
       </c>
       <c r="I56" s="9">
-        <f>ROUND(20*G51*F51,0)</f>
+        <f>ROUND(G24*F56*G56,0)</f>
         <v/>
       </c>
       <c r="J56" s="9">
-        <f>ROUND(H24*F51,0)</f>
+        <f>ROUND(H24*F56,0)</f>
         <v/>
       </c>
       <c r="K56" s="9">
-        <f>ROUND(I24*F51,0)</f>
+        <f>ROUND(I24*F56,0)</f>
         <v/>
       </c>
       <c r="L56" s="46">
-        <f>H51+I51+J51+K51</f>
+        <f>H56+I56+J56+K56</f>
         <v/>
       </c>
     </row>
@@ -13192,31 +13129,32 @@
       <c r="E57" s="44" t="n">
         <v>34354</v>
       </c>
-      <c r="F57" s="170">
-        <f>D52/E52</f>
-        <v/>
-      </c>
-      <c r="G57" s="119" t="n">
-        <v>1505.7</v>
+      <c r="F57" s="188">
+        <f>D57/E57</f>
+        <v/>
+      </c>
+      <c r="G57" s="44">
+        <f>F25</f>
+        <v/>
       </c>
       <c r="H57" s="9">
-        <f>ROUND(D52*G52,0)</f>
+        <f>ROUND(D57*G57,0)</f>
         <v/>
       </c>
       <c r="I57" s="9">
-        <f>ROUND(20*G52*F52,0)</f>
+        <f>ROUND(G25*F57*G57,0)</f>
         <v/>
       </c>
       <c r="J57" s="9">
-        <f>ROUND(H25*F52,0)</f>
+        <f>ROUND(H25*F57,0)</f>
         <v/>
       </c>
       <c r="K57" s="9">
-        <f>ROUND(I25*F52,0)</f>
+        <f>ROUND(I25*F57,0)</f>
         <v/>
       </c>
       <c r="L57" s="46">
-        <f>H52+I52+J52+K52</f>
+        <f>H57+I57+J57+K57</f>
         <v/>
       </c>
     </row>
@@ -13242,31 +13180,32 @@
       <c r="E58" s="44" t="n">
         <v>34354</v>
       </c>
-      <c r="F58" s="170">
-        <f>D53/E53</f>
-        <v/>
-      </c>
-      <c r="G58" s="119" t="n">
-        <v>1505.7</v>
+      <c r="F58" s="188">
+        <f>D58/E58</f>
+        <v/>
+      </c>
+      <c r="G58" s="44">
+        <f>F25</f>
+        <v/>
       </c>
       <c r="H58" s="9">
-        <f>ROUND(D53*G53,0)</f>
+        <f>ROUND(D58*G58,0)</f>
         <v/>
       </c>
       <c r="I58" s="9">
-        <f>ROUND(20*G53*F53,0)</f>
+        <f>ROUND(G25*F58*G58,0)</f>
         <v/>
       </c>
       <c r="J58" s="9">
-        <f>ROUND(H25*F53,0)</f>
+        <f>ROUND(H25*F58,0)</f>
         <v/>
       </c>
       <c r="K58" s="9">
-        <f>ROUND(I25*F53,0)</f>
+        <f>ROUND(I25*F58,0)</f>
         <v/>
       </c>
       <c r="L58" s="46">
-        <f>H53+I53+J53+K53</f>
+        <f>H58+I58+J58+K58</f>
         <v/>
       </c>
     </row>
@@ -13292,31 +13231,32 @@
       <c r="E59" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F59" s="170">
-        <f>D54/E54</f>
-        <v/>
-      </c>
-      <c r="G59" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F59" s="188">
+        <f>D59/E59</f>
+        <v/>
+      </c>
+      <c r="G59" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H59" s="9">
-        <f>ROUND(D54*G54,0)</f>
+        <f>ROUND(D59*G59,0)</f>
         <v/>
       </c>
       <c r="I59" s="9">
-        <f>ROUND(20*G54*F54,0)</f>
+        <f>ROUND(G26*F59*G59,0)</f>
         <v/>
       </c>
       <c r="J59" s="9">
-        <f>ROUND(H26*F54,0)</f>
+        <f>ROUND(H26*F59,0)</f>
         <v/>
       </c>
       <c r="K59" s="9">
-        <f>ROUND(I26*F54,0)</f>
+        <f>ROUND(I26*F59,0)</f>
         <v/>
       </c>
       <c r="L59" s="46">
-        <f>H54+I54+J54+K54</f>
+        <f>H59+I59+J59+K59</f>
         <v/>
       </c>
     </row>
@@ -13342,31 +13282,32 @@
       <c r="E60" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F60" s="170">
-        <f>D55/E55</f>
-        <v/>
-      </c>
-      <c r="G60" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F60" s="188">
+        <f>D60/E60</f>
+        <v/>
+      </c>
+      <c r="G60" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H60" s="9">
-        <f>ROUND(D55*G55,0)</f>
+        <f>ROUND(D60*G60,0)</f>
         <v/>
       </c>
       <c r="I60" s="9">
-        <f>ROUND(20*G55*F55,0)</f>
+        <f>ROUND(G26*F60*G60,0)</f>
         <v/>
       </c>
       <c r="J60" s="9">
-        <f>ROUND(H26*F55,0)</f>
+        <f>ROUND(H26*F60,0)</f>
         <v/>
       </c>
       <c r="K60" s="9">
-        <f>ROUND(I26*F55,0)</f>
+        <f>ROUND(I26*F60,0)</f>
         <v/>
       </c>
       <c r="L60" s="46">
-        <f>H55+I55+J55+K55</f>
+        <f>H60+I60+J60+K60</f>
         <v/>
       </c>
     </row>
@@ -13392,31 +13333,32 @@
       <c r="E61" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F61" s="170">
-        <f>D56/E56</f>
-        <v/>
-      </c>
-      <c r="G61" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F61" s="188">
+        <f>D61/E61</f>
+        <v/>
+      </c>
+      <c r="G61" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H61" s="9">
-        <f>ROUND(D56*G56,0)</f>
+        <f>ROUND(D61*G61,0)</f>
         <v/>
       </c>
       <c r="I61" s="9">
-        <f>ROUND(20*G56*F56,0)</f>
+        <f>ROUND(G26*F61*G61,0)</f>
         <v/>
       </c>
       <c r="J61" s="9">
-        <f>ROUND(H26*F56,0)</f>
+        <f>ROUND(H26*F61,0)</f>
         <v/>
       </c>
       <c r="K61" s="9">
-        <f>ROUND(I26*F56,0)</f>
+        <f>ROUND(I26*F61,0)</f>
         <v/>
       </c>
       <c r="L61" s="46">
-        <f>H56+I56+J56+K56</f>
+        <f>H61+I61+J61+K61</f>
         <v/>
       </c>
     </row>
@@ -13442,31 +13384,32 @@
       <c r="E62" s="44" t="n">
         <v>6553.05</v>
       </c>
-      <c r="F62" s="170">
-        <f>D57/E57</f>
-        <v/>
-      </c>
-      <c r="G62" s="119" t="n">
-        <v>1506.4</v>
+      <c r="F62" s="188">
+        <f>D62/E62</f>
+        <v/>
+      </c>
+      <c r="G62" s="44">
+        <f>F26</f>
+        <v/>
       </c>
       <c r="H62" s="9">
-        <f>ROUND(D57*G57,0)</f>
+        <f>ROUND(D62*G62,0)</f>
         <v/>
       </c>
       <c r="I62" s="9">
-        <f>ROUND(20*G57*F57,0)</f>
+        <f>ROUND(G26*F62*G62,0)</f>
         <v/>
       </c>
       <c r="J62" s="9">
-        <f>ROUND(H26*F57,0)</f>
+        <f>ROUND(H26*F62,0)</f>
         <v/>
       </c>
       <c r="K62" s="9">
-        <f>ROUND(I26*F57,0)</f>
+        <f>ROUND(I26*F62,0)</f>
         <v/>
       </c>
       <c r="L62" s="46">
-        <f>H57+I57+J57+K57</f>
+        <f>H62+I62+J62+K62</f>
         <v/>
       </c>
     </row>
@@ -13492,31 +13435,32 @@
       <c r="E63" s="44" t="n">
         <v>57650</v>
       </c>
-      <c r="F63" s="170">
-        <f>D58/E58</f>
-        <v/>
-      </c>
-      <c r="G63" s="119" t="n">
-        <v>1481.9</v>
+      <c r="F63" s="188">
+        <f>D63/E63</f>
+        <v/>
+      </c>
+      <c r="G63" s="44">
+        <f>F27</f>
+        <v/>
       </c>
       <c r="H63" s="9">
-        <f>ROUND(D58*G58,0)</f>
+        <f>ROUND(D63*G63,0)</f>
         <v/>
       </c>
       <c r="I63" s="9">
-        <f>ROUND(20*G58*F58,0)</f>
+        <f>ROUND(G27*F63*G63,0)</f>
         <v/>
       </c>
       <c r="J63" s="9">
-        <f>ROUND(H27*F58,0)</f>
+        <f>ROUND(H27*F63,0)</f>
         <v/>
       </c>
       <c r="K63" s="9">
-        <f>ROUND(I27*F58,0)</f>
+        <f>ROUND(I27*F63,0)</f>
         <v/>
       </c>
       <c r="L63" s="46">
-        <f>H58+I58+J58+K58</f>
+        <f>H63+I63+J63+K63</f>
         <v/>
       </c>
     </row>
@@ -13542,31 +13486,32 @@
       <c r="E64" s="44" t="n">
         <v>57650</v>
       </c>
-      <c r="F64" s="170">
-        <f>D59/E59</f>
-        <v/>
-      </c>
-      <c r="G64" s="119" t="n">
-        <v>1481.9</v>
+      <c r="F64" s="188">
+        <f>D64/E64</f>
+        <v/>
+      </c>
+      <c r="G64" s="44">
+        <f>F27</f>
+        <v/>
       </c>
       <c r="H64" s="9">
-        <f>ROUND(D59*G59,0)</f>
+        <f>ROUND(D64*G64,0)</f>
         <v/>
       </c>
       <c r="I64" s="9">
-        <f>ROUND(20*G59*F59,0)</f>
+        <f>ROUND(G27*F64*G64,0)</f>
         <v/>
       </c>
       <c r="J64" s="9">
-        <f>ROUND(H27*F59,0)</f>
+        <f>ROUND(H27*F64,0)</f>
         <v/>
       </c>
       <c r="K64" s="9">
-        <f>ROUND(I27*F59,0)</f>
+        <f>ROUND(I27*F64,0)</f>
         <v/>
       </c>
       <c r="L64" s="46">
-        <f>H59+I59+J59+K59</f>
+        <f>H64+I64+J64+K64</f>
         <v/>
       </c>
     </row>
@@ -13592,31 +13537,32 @@
       <c r="E65" s="44" t="n">
         <v>57650</v>
       </c>
-      <c r="F65" s="170">
-        <f>D60/E60</f>
-        <v/>
-      </c>
-      <c r="G65" s="119" t="n">
-        <v>1481.9</v>
+      <c r="F65" s="188">
+        <f>D65/E65</f>
+        <v/>
+      </c>
+      <c r="G65" s="44">
+        <f>F27</f>
+        <v/>
       </c>
       <c r="H65" s="9">
-        <f>ROUND(D60*G60,0)</f>
+        <f>ROUND(D65*G65,0)</f>
         <v/>
       </c>
       <c r="I65" s="9">
-        <f>ROUND(20*G60*F60,0)</f>
+        <f>ROUND(G27*F65*G65,0)</f>
         <v/>
       </c>
       <c r="J65" s="9">
-        <f>ROUND(H27*F60,0)</f>
+        <f>ROUND(H27*F65,0)</f>
         <v/>
       </c>
       <c r="K65" s="9">
-        <f>ROUND(I27*F60,0)</f>
+        <f>ROUND(I27*F65,0)</f>
         <v/>
       </c>
       <c r="L65" s="46">
-        <f>H60+I60+J60+K60</f>
+        <f>H65+I65+J65+K65</f>
         <v/>
       </c>
     </row>
@@ -13642,26 +13588,33 @@
       <c r="E66" s="173" t="n">
         <v>297580</v>
       </c>
-      <c r="F66" s="174" t="n">
-        <v>0.03696484978829222</v>
-      </c>
-      <c r="G66" s="175" t="n">
-        <v>1482.8</v>
-      </c>
-      <c r="H66" s="176" t="n">
-        <v>16310800</v>
-      </c>
-      <c r="I66" s="176" t="n">
-        <v>1096</v>
-      </c>
-      <c r="J66" s="176" t="n">
-        <v>462</v>
-      </c>
-      <c r="K66" s="176" t="n">
-        <v>296</v>
-      </c>
-      <c r="L66" s="177" t="n">
-        <v>16312654</v>
+      <c r="F66" s="189">
+        <f>D66/E66</f>
+        <v/>
+      </c>
+      <c r="G66" s="173">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="H66" s="176">
+        <f>ROUND(D66*G66,0)</f>
+        <v/>
+      </c>
+      <c r="I66" s="176">
+        <f>ROUND(G31*F66*G66,0)</f>
+        <v/>
+      </c>
+      <c r="J66" s="176">
+        <f>ROUND(H31*F66,0)</f>
+        <v/>
+      </c>
+      <c r="K66" s="176">
+        <f>ROUND(I31*F66,0)</f>
+        <v/>
+      </c>
+      <c r="L66" s="177">
+        <f>H66+I66+J66+K66</f>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -13686,26 +13639,33 @@
       <c r="E67" s="173" t="n">
         <v>297580</v>
       </c>
-      <c r="F67" s="174" t="n">
-        <v>0.9630351502117078</v>
-      </c>
-      <c r="G67" s="175" t="n">
-        <v>1482.8</v>
-      </c>
-      <c r="H67" s="176" t="n">
-        <v>424990980</v>
-      </c>
-      <c r="I67" s="176" t="n">
-        <v>28560</v>
-      </c>
-      <c r="J67" s="176" t="n">
-        <v>12038</v>
-      </c>
-      <c r="K67" s="176" t="n">
-        <v>7704</v>
-      </c>
-      <c r="L67" s="177" t="n">
-        <v>425039282</v>
+      <c r="F67" s="189">
+        <f>D67/E67</f>
+        <v/>
+      </c>
+      <c r="G67" s="173">
+        <f>F31</f>
+        <v/>
+      </c>
+      <c r="H67" s="176">
+        <f>ROUND(D67*G67,0)</f>
+        <v/>
+      </c>
+      <c r="I67" s="176">
+        <f>ROUND(G31*F67*G67,0)</f>
+        <v/>
+      </c>
+      <c r="J67" s="176">
+        <f>ROUND(H31*F67,0)</f>
+        <v/>
+      </c>
+      <c r="K67" s="176">
+        <f>ROUND(I31*F67,0)</f>
+        <v/>
+      </c>
+      <c r="L67" s="177">
+        <f>H67+I67+J67+K67</f>
+        <v/>
       </c>
     </row>
     <row r="68">
@@ -13730,26 +13690,33 @@
       <c r="E68" s="173" t="n">
         <v>4388.4</v>
       </c>
-      <c r="F68" s="174" t="n">
-        <v>1</v>
-      </c>
-      <c r="G68" s="175" t="n">
-        <v>1741.08</v>
-      </c>
-      <c r="H68" s="176" t="n">
-        <v>7702082</v>
-      </c>
-      <c r="I68" s="176" t="n">
-        <v>43527</v>
-      </c>
-      <c r="J68" s="176" t="n">
-        <v>10000</v>
-      </c>
-      <c r="K68" s="176" t="n">
-        <v>8000</v>
-      </c>
-      <c r="L68" s="177" t="n">
-        <v>7763609</v>
+      <c r="F68" s="189">
+        <f>D68/E68</f>
+        <v/>
+      </c>
+      <c r="G68" s="173">
+        <f>F32</f>
+        <v/>
+      </c>
+      <c r="H68" s="176">
+        <f>ROUND(D68*G68,0)</f>
+        <v/>
+      </c>
+      <c r="I68" s="176">
+        <f>ROUND(G32*F68*G68,0)</f>
+        <v/>
+      </c>
+      <c r="J68" s="176">
+        <f>ROUND(H32*F68,0)</f>
+        <v/>
+      </c>
+      <c r="K68" s="176">
+        <f>ROUND(I32*F68,0)</f>
+        <v/>
+      </c>
+      <c r="L68" s="177">
+        <f>H68+I68+J68+K68</f>
+        <v/>
       </c>
     </row>
     <row r="76">

</xml_diff>

<commit_message>
Fix tariff comments: remove from CPO682 (84170), add to CPO683 (0) (19:35)
</commit_message>
<xml_diff>
--- a/RNR_수입원가_2026_20260424.xlsx
+++ b/RNR_수입원가_2026_20260424.xlsx
@@ -979,10 +979,11 @@
 (정보기술협정 양허품목)</t>
       </text>
     </comment>
-    <comment ref="S13" authorId="0" shapeId="0">
+    <comment ref="S14" authorId="0" shapeId="0">
       <text>
         <t>ITA(정보기술협정) 관세면제
-HS 8518/8543 디지털시네마장비</t>
+HS 8414.59 — Projector cooling fan
+(WTO 협정세율 0%)</t>
       </text>
     </comment>
     <comment ref="S15" authorId="0" shapeId="0">

</xml_diff>